<commit_message>
Research: 25-stock robotics/autonomy basket from ARKQ+BOTZ; BOTZ rebuilt with Keyence (parser fix)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kn9FvRUhfk3FShXDYTTURS
</commit_message>
<xml_diff>
--- a/research/index-studies/BOTZ_Weights_PE_Sales.xlsx
+++ b/research/index-studies/BOTZ_Weights_PE_Sales.xlsx
@@ -16,7 +16,7 @@
     <sheet name="By Decade" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Holdings!$A$1:$N$80</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Holdings!$A$1:$N$81</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="298">
   <si>
     <t xml:space="preserve">Rank</t>
   </si>
@@ -123,6 +123,15 @@
     <t xml:space="preserve">Semiconductors</t>
   </si>
   <si>
+    <t xml:space="preserve">6861</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keyence Corporation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scientific &amp; Technical Instruments</t>
+  </si>
+  <si>
     <t xml:space="preserve">6273</t>
   </si>
   <si>
@@ -165,9 +174,6 @@
     <t xml:space="preserve">Cognex Corporation</t>
   </si>
   <si>
-    <t xml:space="preserve">Scientific &amp; Technical Instruments</t>
-  </si>
-  <si>
     <t xml:space="preserve">TSLA</t>
   </si>
   <si>
@@ -510,12 +516,6 @@
     <t xml:space="preserve">CiDi Inc.</t>
   </si>
   <si>
-    <t xml:space="preserve">NQZ6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NASDAQ 100 E-MINI DEC26</t>
-  </si>
-  <si>
     <t xml:space="preserve">2590</t>
   </si>
   <si>
@@ -555,7 +555,7 @@
     <t xml:space="preserve">MOG/A</t>
   </si>
   <si>
-    <t xml:space="preserve">MOOG INC-CLASS A</t>
+    <t xml:space="preserve">Moog Inc.</t>
   </si>
   <si>
     <t xml:space="preserve">AVEX</t>
@@ -648,6 +648,12 @@
     <t xml:space="preserve">Integrated Freight &amp; Logistics</t>
   </si>
   <si>
+    <t xml:space="preserve">348340</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neuromeka Co Ltd</t>
+  </si>
+  <si>
     <t xml:space="preserve">RR</t>
   </si>
   <si>
@@ -714,7 +720,7 @@
     <t xml:space="preserve">Holdings shared with the S&amp;P 500 (S&amp;P weights from the companion S&amp;P 500 workbook, Sept 2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">6 of 79 holdings are S&amp;P 500 members</t>
+    <t xml:space="preserve">6 of 80 holdings are S&amp;P 500 members</t>
   </si>
   <si>
     <t xml:space="preserve">Share of this fund's weight that is inside the S&amp;P 500</t>
@@ -1484,7 +1490,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N80"/>
+  <dimension ref="A1:N81"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.99"/>
@@ -1564,11 +1570,11 @@
         <v>17</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.091285</v>
+        <v>0.084381</v>
       </c>
       <c r="G2" s="3" t="n">
         <f aca="false">SUM($F$2:F2)</f>
-        <v>0.091285</v>
+        <v>0.084381</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>398.3</v>
@@ -1608,11 +1614,11 @@
         <v>21</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.089762</v>
+        <v>0.082973</v>
       </c>
       <c r="G3" s="3" t="n">
         <f aca="false">SUM($F$2:F3)</f>
-        <v>0.181047</v>
+        <v>0.167354</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="5" t="n">
@@ -1650,11 +1656,11 @@
         <v>25</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.08715</v>
+        <v>0.080559</v>
       </c>
       <c r="G4" s="3" t="n">
         <f aca="false">SUM($F$2:F4)</f>
-        <v>0.268197</v>
+        <v>0.247913</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="5" t="n">
@@ -1692,11 +1698,11 @@
         <v>30</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.086171</v>
+        <v>0.079654</v>
       </c>
       <c r="G5" s="3" t="n">
         <f aca="false">SUM($F$2:F5)</f>
-        <v>0.354368</v>
+        <v>0.327567</v>
       </c>
       <c r="H5" s="4" t="n">
         <v>225.51</v>
@@ -1730,28 +1736,28 @@
         <v>32</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.048091</v>
+        <v>0.077643</v>
       </c>
       <c r="G6" s="3" t="n">
         <f aca="false">SUM($F$2:F6)</f>
-        <v>0.402459</v>
+        <v>0.40521</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="5" t="n">
-        <v>25.7545</v>
+        <v>42.0421</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2639.93</v>
+        <v>1837.92</v>
       </c>
       <c r="K6" s="5"/>
       <c r="L6" s="6" t="n">
-        <v>4.6509</v>
+        <v>14.9342</v>
       </c>
       <c r="M6" s="5" t="str">
         <f aca="false">IF(AND(N(K6)&gt;0,N(L6)&gt;0),K6/L6,"")</f>
@@ -1766,10 +1772,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>20</v>
@@ -1778,22 +1784,22 @@
         <v>25</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.035578</v>
+        <v>0.044453</v>
       </c>
       <c r="G7" s="3" t="n">
         <f aca="false">SUM($F$2:F7)</f>
-        <v>0.438037</v>
+        <v>0.449663</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="5" t="n">
-        <v>25.5268</v>
+        <v>25.7545</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>216.87</v>
+        <v>2639.93</v>
       </c>
       <c r="K7" s="5"/>
       <c r="L7" s="6" t="n">
-        <v>2.9844</v>
+        <v>4.6509</v>
       </c>
       <c r="M7" s="5" t="str">
         <f aca="false">IF(AND(N(K7)&gt;0,N(L7)&gt;0),K7/L7,"")</f>
@@ -1808,43 +1814,41 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.030029</v>
+        <v>0.032887</v>
       </c>
       <c r="G8" s="3" t="n">
         <f aca="false">SUM($F$2:F8)</f>
-        <v>0.468066</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>6.32</v>
-      </c>
-      <c r="I8" s="5"/>
+        <v>0.48255</v>
+      </c>
+      <c r="H8" s="4"/>
+      <c r="I8" s="5" t="n">
+        <v>25.5268</v>
+      </c>
       <c r="J8" s="4" t="n">
-        <v>-0.46</v>
-      </c>
-      <c r="K8" s="5" t="n">
-        <v>12.6663</v>
-      </c>
+        <v>216.87</v>
+      </c>
+      <c r="K8" s="5"/>
       <c r="L8" s="6" t="n">
-        <v>2533.2522</v>
-      </c>
-      <c r="M8" s="5" t="n">
+        <v>2.9844</v>
+      </c>
+      <c r="M8" s="5" t="str">
         <f aca="false">IF(AND(N(K8)&gt;0,N(L8)&gt;0),K8/L8,"")</f>
-        <v>0.0050000153952299</v>
+        <v/>
       </c>
       <c r="N8" s="2" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1852,38 +1856,40 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="F9" s="3" t="n">
-        <v>0.028071</v>
+        <v>0.027758</v>
       </c>
       <c r="G9" s="3" t="n">
         <f aca="false">SUM($F$2:F9)</f>
-        <v>0.496137</v>
-      </c>
-      <c r="H9" s="4"/>
-      <c r="I9" s="5" t="n">
-        <v>29.618</v>
-      </c>
+        <v>0.510308</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="I9" s="5"/>
       <c r="J9" s="4" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="K9" s="5"/>
+        <v>-0.46</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>12.6663</v>
+      </c>
       <c r="L9" s="6" t="n">
-        <v>2.8995</v>
-      </c>
-      <c r="M9" s="5" t="str">
+        <v>2533.2522</v>
+      </c>
+      <c r="M9" s="5" t="n">
         <f aca="false">IF(AND(N(K9)&gt;0,N(L9)&gt;0),K9/L9,"")</f>
-        <v/>
+        <v>0.0050000153952299</v>
       </c>
       <c r="N9" s="2" t="s">
         <v>42</v>
@@ -1900,38 +1906,36 @@
         <v>44</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.026983</v>
+        <v>0.025948</v>
       </c>
       <c r="G10" s="3" t="n">
         <f aca="false">SUM($F$2:F10)</f>
-        <v>0.52312</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>58.19</v>
-      </c>
+        <v>0.536256</v>
+      </c>
+      <c r="H10" s="4"/>
       <c r="I10" s="5" t="n">
-        <v>55.9519</v>
+        <v>29.618</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="K10" s="5" t="n">
-        <v>9.7889</v>
-      </c>
+        <v>1.78</v>
+      </c>
+      <c r="K10" s="5"/>
       <c r="L10" s="6" t="n">
-        <v>8.9895</v>
-      </c>
-      <c r="M10" s="5" t="n">
+        <v>2.8995</v>
+      </c>
+      <c r="M10" s="5" t="str">
         <f aca="false">IF(AND(N(K10)&gt;0,N(L10)&gt;0),K10/L10,"")</f>
-        <v>1.08892596918627</v>
-      </c>
-      <c r="N10" s="2"/>
+        <v/>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="n">
@@ -1944,36 +1948,36 @@
         <v>47</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.022413</v>
+        <v>0.024942</v>
       </c>
       <c r="G11" s="3" t="n">
         <f aca="false">SUM($F$2:F11)</f>
-        <v>0.545533</v>
+        <v>0.561198</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>380.12</v>
+        <v>58.19</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>345.5636</v>
+        <v>55.9519</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>1.1</v>
+        <v>1.04</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>1501.302</v>
+        <v>9.7889</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>14.4887</v>
+        <v>8.9895</v>
       </c>
       <c r="M11" s="5" t="n">
         <f aca="false">IF(AND(N(K11)&gt;0,N(L11)&gt;0),K11/L11,"")</f>
-        <v>103.618820184005</v>
+        <v>1.08892596918627</v>
       </c>
       <c r="N11" s="2"/>
     </row>
@@ -1982,42 +1986,42 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="F12" s="3" t="n">
-        <v>0.021978</v>
+        <v>0.020718</v>
       </c>
       <c r="G12" s="3" t="n">
         <f aca="false">SUM($F$2:F12)</f>
-        <v>0.567511</v>
+        <v>0.581916</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>337.83</v>
+        <v>380.12</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>16.9338</v>
+        <v>345.5636</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>19.95</v>
+        <v>1.1</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>4131.6387</v>
+        <v>1501.302</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>9.2665</v>
+        <v>14.4887</v>
       </c>
       <c r="M12" s="5" t="n">
         <f aca="false">IF(AND(N(K12)&gt;0,N(L12)&gt;0),K12/L12,"")</f>
-        <v>445.868310581126</v>
+        <v>103.618820184005</v>
       </c>
       <c r="N12" s="2"/>
     </row>
@@ -2026,81 +2030,83 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="F13" s="3" t="n">
-        <v>0.021978</v>
+        <v>0.020316</v>
       </c>
       <c r="G13" s="3" t="n">
         <f aca="false">SUM($F$2:F13)</f>
-        <v>0.589489</v>
-      </c>
-      <c r="H13" s="4"/>
-      <c r="I13" s="5"/>
+        <v>0.602232</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>337.83</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>16.9338</v>
+      </c>
       <c r="J13" s="4" t="n">
-        <v>-0.18</v>
-      </c>
-      <c r="K13" s="5"/>
+        <v>19.95</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>4131.6387</v>
+      </c>
       <c r="L13" s="6" t="n">
-        <v>76.5233</v>
-      </c>
-      <c r="M13" s="5" t="str">
+        <v>9.2665</v>
+      </c>
+      <c r="M13" s="5" t="n">
         <f aca="false">IF(AND(N(K13)&gt;0,N(L13)&gt;0),K13/L13,"")</f>
-        <v/>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>55</v>
-      </c>
+        <v>445.868310581126</v>
+      </c>
+      <c r="N13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="D14" s="2" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.021869</v>
+        <v>0.020316</v>
       </c>
       <c r="G14" s="3" t="n">
         <f aca="false">SUM($F$2:F14)</f>
-        <v>0.611358</v>
+        <v>0.622548</v>
       </c>
       <c r="H14" s="4"/>
-      <c r="I14" s="5" t="n">
-        <v>36.3401</v>
-      </c>
+      <c r="I14" s="5"/>
       <c r="J14" s="4" t="n">
-        <v>173.94</v>
+        <v>-0.18</v>
       </c>
       <c r="K14" s="5"/>
       <c r="L14" s="6" t="n">
-        <v>1.533</v>
+        <v>76.5233</v>
       </c>
       <c r="M14" s="5" t="str">
         <f aca="false">IF(AND(N(K14)&gt;0,N(L14)&gt;0),K14/L14,"")</f>
         <v/>
       </c>
       <c r="N14" s="2" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2108,86 +2114,86 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="F15" s="3" t="n">
-        <v>0.021216</v>
+        <v>0.020215</v>
       </c>
       <c r="G15" s="3" t="n">
         <f aca="false">SUM($F$2:F15)</f>
-        <v>0.632574</v>
-      </c>
-      <c r="H15" s="4" t="n">
-        <v>709.48</v>
-      </c>
+        <v>0.642763</v>
+      </c>
+      <c r="H15" s="4"/>
       <c r="I15" s="5" t="n">
-        <v>39.4156</v>
+        <v>36.3401</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="K15" s="5" t="n">
-        <v>191.2938</v>
-      </c>
+        <v>173.94</v>
+      </c>
+      <c r="K15" s="5"/>
       <c r="L15" s="6" t="n">
-        <v>3.9914</v>
-      </c>
-      <c r="M15" s="5" t="n">
+        <v>1.533</v>
+      </c>
+      <c r="M15" s="5" t="str">
         <f aca="false">IF(AND(N(K15)&gt;0,N(L15)&gt;0),K15/L15,"")</f>
-        <v>47.9264919577091</v>
-      </c>
-      <c r="N15" s="2"/>
+        <v/>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>21</v>
+        <v>63</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.020128</v>
+        <v>0.019612</v>
       </c>
       <c r="G16" s="3" t="n">
         <f aca="false">SUM($F$2:F16)</f>
-        <v>0.652702</v>
-      </c>
-      <c r="H16" s="4"/>
+        <v>0.662375</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>709.48</v>
+      </c>
       <c r="I16" s="5" t="n">
-        <v>32.9653</v>
+        <v>39.4156</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>135.87</v>
-      </c>
-      <c r="K16" s="5"/>
+        <v>18</v>
+      </c>
+      <c r="K16" s="5" t="n">
+        <v>191.2938</v>
+      </c>
       <c r="L16" s="6" t="n">
-        <v>2.0914</v>
-      </c>
-      <c r="M16" s="5" t="str">
+        <v>3.9914</v>
+      </c>
+      <c r="M16" s="5" t="n">
         <f aca="false">IF(AND(N(K16)&gt;0,N(L16)&gt;0),K16/L16,"")</f>
-        <v/>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>26</v>
-      </c>
+        <v>47.9264919577091</v>
+      </c>
+      <c r="N16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="n">
@@ -2200,33 +2206,35 @@
         <v>65</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>66</v>
+        <v>21</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>0.019584</v>
+        <v>0.018606</v>
       </c>
       <c r="G17" s="3" t="n">
         <f aca="false">SUM($F$2:F17)</f>
-        <v>0.672286</v>
+        <v>0.680981</v>
       </c>
       <c r="H17" s="4"/>
-      <c r="I17" s="5"/>
+      <c r="I17" s="5" t="n">
+        <v>32.9653</v>
+      </c>
       <c r="J17" s="4" t="n">
-        <v>-0.73</v>
+        <v>135.87</v>
       </c>
       <c r="K17" s="5"/>
       <c r="L17" s="6" t="n">
-        <v>14.8982</v>
+        <v>2.0914</v>
       </c>
       <c r="M17" s="5" t="str">
         <f aca="false">IF(AND(N(K17)&gt;0,N(L17)&gt;0),K17/L17,"")</f>
         <v/>
       </c>
       <c r="N17" s="2" t="s">
-        <v>67</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2234,41 +2242,39 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>29</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>0.017517</v>
+        <v>0.018103</v>
       </c>
       <c r="G18" s="3" t="n">
         <f aca="false">SUM($F$2:F18)</f>
-        <v>0.689803</v>
+        <v>0.699084</v>
       </c>
       <c r="H18" s="4"/>
-      <c r="I18" s="5" t="n">
-        <v>18.2517</v>
-      </c>
+      <c r="I18" s="5"/>
       <c r="J18" s="4" t="n">
-        <v>1.43</v>
+        <v>-0.73</v>
       </c>
       <c r="K18" s="5"/>
       <c r="L18" s="6" t="n">
-        <v>1.5324</v>
+        <v>14.8982</v>
       </c>
       <c r="M18" s="5" t="str">
         <f aca="false">IF(AND(N(K18)&gt;0,N(L18)&gt;0),K18/L18,"")</f>
         <v/>
       </c>
       <c r="N18" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2276,31 +2282,41 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
       <c r="F19" s="3" t="n">
-        <v>0.017082</v>
+        <v>0.016192</v>
       </c>
       <c r="G19" s="3" t="n">
         <f aca="false">SUM($F$2:F19)</f>
-        <v>0.706885</v>
+        <v>0.715276</v>
       </c>
       <c r="H19" s="4"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="4"/>
+      <c r="I19" s="5" t="n">
+        <v>18.2517</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>1.43</v>
+      </c>
       <c r="K19" s="5"/>
-      <c r="L19" s="6"/>
+      <c r="L19" s="6" t="n">
+        <v>1.5324</v>
+      </c>
       <c r="M19" s="5" t="str">
         <f aca="false">IF(AND(N(K19)&gt;0,N(L19)&gt;0),K19/L19,"")</f>
         <v/>
       </c>
       <c r="N19" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2308,45 +2324,31 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
       <c r="F20" s="3" t="n">
-        <v>0.015885</v>
+        <v>0.01579</v>
       </c>
       <c r="G20" s="3" t="n">
         <f aca="false">SUM($F$2:F20)</f>
-        <v>0.72277</v>
-      </c>
-      <c r="H20" s="4" t="n">
-        <v>43.69</v>
-      </c>
-      <c r="I20" s="5" t="n">
-        <v>1092.25</v>
-      </c>
-      <c r="J20" s="4" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="K20" s="5" t="n">
-        <v>26.4484</v>
-      </c>
-      <c r="L20" s="6" t="n">
-        <v>9.9965</v>
-      </c>
-      <c r="M20" s="5" t="n">
+        <v>0.731066</v>
+      </c>
+      <c r="H20" s="4"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="6"/>
+      <c r="M20" s="5" t="str">
         <f aca="false">IF(AND(N(K20)&gt;0,N(L20)&gt;0),K20/L20,"")</f>
-        <v>2.64576601810634</v>
+        <v/>
       </c>
       <c r="N20" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2354,10 +2356,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>20</v>
@@ -2366,29 +2368,33 @@
         <v>25</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0.015776</v>
+        <v>0.014684</v>
       </c>
       <c r="G21" s="3" t="n">
         <f aca="false">SUM($F$2:F21)</f>
-        <v>0.738546</v>
-      </c>
-      <c r="H21" s="4"/>
+        <v>0.74575</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>43.69</v>
+      </c>
       <c r="I21" s="5" t="n">
-        <v>35.3778</v>
+        <v>1092.25</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="K21" s="5"/>
+        <v>0.04</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>26.4484</v>
+      </c>
       <c r="L21" s="6" t="n">
-        <v>78.9726</v>
-      </c>
-      <c r="M21" s="5" t="str">
+        <v>9.9965</v>
+      </c>
+      <c r="M21" s="5" t="n">
         <f aca="false">IF(AND(N(K21)&gt;0,N(L21)&gt;0),K21/L21,"")</f>
-        <v/>
+        <v>2.64576601810634</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2396,10 +2402,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>20</v>
@@ -2408,27 +2414,29 @@
         <v>25</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>0.012186</v>
+        <v>0.014583</v>
       </c>
       <c r="G22" s="3" t="n">
         <f aca="false">SUM($F$2:F22)</f>
-        <v>0.750732</v>
+        <v>0.760333</v>
       </c>
       <c r="H22" s="4"/>
-      <c r="I22" s="5"/>
+      <c r="I22" s="5" t="n">
+        <v>35.3778</v>
+      </c>
       <c r="J22" s="4" t="n">
-        <v>-1.44</v>
+        <v>0.45</v>
       </c>
       <c r="K22" s="5"/>
       <c r="L22" s="6" t="n">
-        <v>15.0241</v>
+        <v>78.9726</v>
       </c>
       <c r="M22" s="5" t="str">
         <f aca="false">IF(AND(N(K22)&gt;0,N(L22)&gt;0),K22/L22,"")</f>
         <v/>
       </c>
       <c r="N22" s="2" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2448,29 +2456,27 @@
         <v>25</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>0.012186</v>
+        <v>0.011264</v>
       </c>
       <c r="G23" s="3" t="n">
         <f aca="false">SUM($F$2:F23)</f>
-        <v>0.762918</v>
+        <v>0.771597</v>
       </c>
       <c r="H23" s="4"/>
-      <c r="I23" s="5" t="n">
-        <v>41.2788</v>
-      </c>
+      <c r="I23" s="5"/>
       <c r="J23" s="4" t="n">
-        <v>178.76</v>
+        <v>-1.44</v>
       </c>
       <c r="K23" s="5"/>
       <c r="L23" s="6" t="n">
-        <v>3.2481</v>
+        <v>15.0241</v>
       </c>
       <c r="M23" s="5" t="str">
         <f aca="false">IF(AND(N(K23)&gt;0,N(L23)&gt;0),K23/L23,"")</f>
         <v/>
       </c>
       <c r="N23" s="2" t="s">
-        <v>26</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2490,29 +2496,29 @@
         <v>25</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>0.011424</v>
+        <v>0.011264</v>
       </c>
       <c r="G24" s="3" t="n">
         <f aca="false">SUM($F$2:F24)</f>
-        <v>0.774342</v>
+        <v>0.782861</v>
       </c>
       <c r="H24" s="4"/>
       <c r="I24" s="5" t="n">
-        <v>372.5974</v>
+        <v>41.2788</v>
       </c>
       <c r="J24" s="4" t="n">
-        <v>0.77</v>
+        <v>178.76</v>
       </c>
       <c r="K24" s="5"/>
       <c r="L24" s="6" t="n">
-        <v>78.7562</v>
+        <v>3.2481</v>
       </c>
       <c r="M24" s="5" t="str">
         <f aca="false">IF(AND(N(K24)&gt;0,N(L24)&gt;0),K24/L24,"")</f>
         <v/>
       </c>
       <c r="N24" s="2" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2532,32 +2538,30 @@
         <v>25</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>0.011207</v>
+        <v>0.01056</v>
       </c>
       <c r="G25" s="3" t="n">
         <f aca="false">SUM($F$2:F25)</f>
-        <v>0.785549</v>
-      </c>
-      <c r="H25" s="4" t="n">
-        <v>432.89</v>
-      </c>
+        <v>0.793421</v>
+      </c>
+      <c r="H25" s="4"/>
       <c r="I25" s="5" t="n">
-        <v>40.5328</v>
+        <v>372.5974</v>
       </c>
       <c r="J25" s="4" t="n">
-        <v>10.68</v>
-      </c>
-      <c r="K25" s="5" t="n">
-        <v>48.1694</v>
-      </c>
+        <v>0.77</v>
+      </c>
+      <c r="K25" s="5"/>
       <c r="L25" s="6" t="n">
-        <v>5.3683</v>
-      </c>
-      <c r="M25" s="5" t="n">
+        <v>78.7562</v>
+      </c>
+      <c r="M25" s="5" t="str">
         <f aca="false">IF(AND(N(K25)&gt;0,N(L25)&gt;0),K25/L25,"")</f>
-        <v>8.97293370340704</v>
-      </c>
-      <c r="N25" s="2"/>
+        <v/>
+      </c>
+      <c r="N25" s="2" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="n">
@@ -2576,30 +2580,32 @@
         <v>25</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>0.010336</v>
+        <v>0.010359</v>
       </c>
       <c r="G26" s="3" t="n">
         <f aca="false">SUM($F$2:F26)</f>
-        <v>0.795885</v>
-      </c>
-      <c r="H26" s="4"/>
+        <v>0.80378</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>432.89</v>
+      </c>
       <c r="I26" s="5" t="n">
-        <v>375.7467</v>
+        <v>40.5328</v>
       </c>
       <c r="J26" s="4" t="n">
-        <v>16.74</v>
-      </c>
-      <c r="K26" s="5"/>
+        <v>10.68</v>
+      </c>
+      <c r="K26" s="5" t="n">
+        <v>48.1694</v>
+      </c>
       <c r="L26" s="6" t="n">
-        <v>9.4905</v>
-      </c>
-      <c r="M26" s="5" t="str">
+        <v>5.3683</v>
+      </c>
+      <c r="M26" s="5" t="n">
         <f aca="false">IF(AND(N(K26)&gt;0,N(L26)&gt;0),K26/L26,"")</f>
-        <v/>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>26</v>
-      </c>
+        <v>8.97293370340704</v>
+      </c>
+      <c r="N26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="n">
@@ -2615,32 +2621,32 @@
         <v>20</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>0.01001</v>
+        <v>0.009554</v>
       </c>
       <c r="G27" s="3" t="n">
         <f aca="false">SUM($F$2:F27)</f>
-        <v>0.805895</v>
+        <v>0.813334</v>
       </c>
       <c r="H27" s="4"/>
       <c r="I27" s="5" t="n">
-        <v>49.0152</v>
+        <v>375.7467</v>
       </c>
       <c r="J27" s="4" t="n">
-        <v>6.6</v>
+        <v>16.74</v>
       </c>
       <c r="K27" s="5"/>
       <c r="L27" s="6" t="n">
-        <v>4.3376</v>
+        <v>9.4905</v>
       </c>
       <c r="M27" s="5" t="str">
         <f aca="false">IF(AND(N(K27)&gt;0,N(L27)&gt;0),K27/L27,"")</f>
         <v/>
       </c>
       <c r="N27" s="2" t="s">
-        <v>94</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2648,37 +2654,41 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>25</v>
+        <v>95</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>0.009248</v>
+        <v>0.009253</v>
       </c>
       <c r="G28" s="3" t="n">
         <f aca="false">SUM($F$2:F28)</f>
-        <v>0.815143</v>
+        <v>0.822587</v>
       </c>
       <c r="H28" s="4"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="4"/>
+      <c r="I28" s="5" t="n">
+        <v>49.0152</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>6.6</v>
+      </c>
       <c r="K28" s="5"/>
       <c r="L28" s="6" t="n">
-        <v>81.7533</v>
+        <v>4.3376</v>
       </c>
       <c r="M28" s="5" t="str">
         <f aca="false">IF(AND(N(K28)&gt;0,N(L28)&gt;0),K28/L28,"")</f>
         <v/>
       </c>
       <c r="N28" s="2" t="s">
-        <v>74</v>
+        <v>96</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2692,33 +2702,31 @@
         <v>98</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>0.009248</v>
+        <v>0.008549</v>
       </c>
       <c r="G29" s="3" t="n">
         <f aca="false">SUM($F$2:F29)</f>
-        <v>0.824391</v>
+        <v>0.831136</v>
       </c>
       <c r="H29" s="4"/>
       <c r="I29" s="5"/>
-      <c r="J29" s="4" t="n">
-        <v>-9.16</v>
-      </c>
+      <c r="J29" s="4"/>
       <c r="K29" s="5"/>
       <c r="L29" s="6" t="n">
-        <v>3.0828</v>
+        <v>81.7533</v>
       </c>
       <c r="M29" s="5" t="str">
         <f aca="false">IF(AND(N(K29)&gt;0,N(L29)&gt;0),K29/L29,"")</f>
         <v/>
       </c>
       <c r="N29" s="2" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2726,31 +2734,39 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
+      <c r="D30" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="F30" s="3" t="n">
-        <v>0.008813</v>
+        <v>0.008549</v>
       </c>
       <c r="G30" s="3" t="n">
         <f aca="false">SUM($F$2:F30)</f>
-        <v>0.833204</v>
+        <v>0.839685</v>
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="5"/>
-      <c r="J30" s="4"/>
+      <c r="J30" s="4" t="n">
+        <v>-9.16</v>
+      </c>
       <c r="K30" s="5"/>
-      <c r="L30" s="6"/>
+      <c r="L30" s="6" t="n">
+        <v>3.0828</v>
+      </c>
       <c r="M30" s="5" t="str">
         <f aca="false">IF(AND(N(K30)&gt;0,N(L30)&gt;0),K30/L30,"")</f>
         <v/>
       </c>
       <c r="N30" s="2" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2763,38 +2779,26 @@
       <c r="C31" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>58</v>
-      </c>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
       <c r="F31" s="3" t="n">
-        <v>0.007943</v>
+        <v>0.008146</v>
       </c>
       <c r="G31" s="3" t="n">
         <f aca="false">SUM($F$2:F31)</f>
-        <v>0.841147</v>
-      </c>
-      <c r="H31" s="4" t="n">
-        <v>39.38</v>
-      </c>
+        <v>0.847831</v>
+      </c>
+      <c r="H31" s="4"/>
       <c r="I31" s="5"/>
-      <c r="J31" s="4" t="n">
-        <v>-0.83</v>
-      </c>
-      <c r="K31" s="5" t="n">
-        <v>2.8398</v>
-      </c>
-      <c r="L31" s="6" t="n">
-        <v>13.8589</v>
-      </c>
-      <c r="M31" s="5" t="n">
+      <c r="J31" s="4"/>
+      <c r="K31" s="5"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="5" t="str">
         <f aca="false">IF(AND(N(K31)&gt;0,N(L31)&gt;0),K31/L31,"")</f>
-        <v>0.204908037434428</v>
+        <v/>
       </c>
       <c r="N31" s="2" t="s">
-        <v>39</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2811,34 +2815,34 @@
         <v>29</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>106</v>
+        <v>60</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>0.006963</v>
+        <v>0.007342</v>
       </c>
       <c r="G32" s="3" t="n">
         <f aca="false">SUM($F$2:F32)</f>
-        <v>0.84811</v>
+        <v>0.855173</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>7.26</v>
+        <v>39.38</v>
       </c>
       <c r="I32" s="5"/>
       <c r="J32" s="4" t="n">
-        <v>-0.33</v>
+        <v>-0.83</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>3.1538</v>
+        <v>2.8398</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>25.2233</v>
+        <v>13.8589</v>
       </c>
       <c r="M32" s="5" t="n">
         <f aca="false">IF(AND(N(K32)&gt;0,N(L32)&gt;0),K32/L32,"")</f>
-        <v>0.125035185721139</v>
+        <v>0.204908037434428</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2846,39 +2850,43 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="D33" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="D33" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="F33" s="3" t="n">
-        <v>0.006855</v>
+        <v>0.006437</v>
       </c>
       <c r="G33" s="3" t="n">
         <f aca="false">SUM($F$2:F33)</f>
-        <v>0.854965</v>
-      </c>
-      <c r="H33" s="4"/>
+        <v>0.86161</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>7.26</v>
+      </c>
       <c r="I33" s="5"/>
       <c r="J33" s="4" t="n">
-        <v>-0.28</v>
-      </c>
-      <c r="K33" s="5"/>
+        <v>-0.33</v>
+      </c>
+      <c r="K33" s="5" t="n">
+        <v>3.1538</v>
+      </c>
       <c r="L33" s="6" t="n">
-        <v>39.6386</v>
-      </c>
-      <c r="M33" s="5" t="str">
+        <v>25.2233</v>
+      </c>
+      <c r="M33" s="5" t="n">
         <f aca="false">IF(AND(N(K33)&gt;0,N(L33)&gt;0),K33/L33,"")</f>
-        <v/>
+        <v>0.125035185721139</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>67</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2886,41 +2894,39 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="D34" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>112</v>
-      </c>
       <c r="F34" s="3" t="n">
-        <v>0.006528</v>
+        <v>0.006336</v>
       </c>
       <c r="G34" s="3" t="n">
         <f aca="false">SUM($F$2:F34)</f>
-        <v>0.861493</v>
+        <v>0.867946</v>
       </c>
       <c r="H34" s="4"/>
-      <c r="I34" s="5" t="n">
-        <v>735.2941</v>
-      </c>
+      <c r="I34" s="5"/>
       <c r="J34" s="4" t="n">
-        <v>0.17</v>
+        <v>-0.28</v>
       </c>
       <c r="K34" s="5"/>
       <c r="L34" s="6" t="n">
-        <v>4.219</v>
+        <v>39.6386</v>
       </c>
       <c r="M34" s="5" t="str">
         <f aca="false">IF(AND(N(K34)&gt;0,N(L34)&gt;0),K34/L34,"")</f>
         <v/>
       </c>
       <c r="N34" s="2" t="s">
-        <v>113</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2928,41 +2934,41 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>25</v>
+        <v>114</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>0.006528</v>
+        <v>0.006034</v>
       </c>
       <c r="G35" s="3" t="n">
         <f aca="false">SUM($F$2:F35)</f>
-        <v>0.868021</v>
+        <v>0.87398</v>
       </c>
       <c r="H35" s="4"/>
       <c r="I35" s="5" t="n">
-        <v>17.9322</v>
+        <v>735.2941</v>
       </c>
       <c r="J35" s="4" t="n">
-        <v>6.49</v>
+        <v>0.17</v>
       </c>
       <c r="K35" s="5"/>
       <c r="L35" s="6" t="n">
-        <v>1.447</v>
+        <v>4.219</v>
       </c>
       <c r="M35" s="5" t="str">
         <f aca="false">IF(AND(N(K35)&gt;0,N(L35)&gt;0),K35/L35,"")</f>
         <v/>
       </c>
       <c r="N35" s="2" t="s">
-        <v>42</v>
+        <v>115</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2976,35 +2982,35 @@
         <v>117</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>118</v>
+        <v>25</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>0.006311</v>
+        <v>0.006034</v>
       </c>
       <c r="G36" s="3" t="n">
         <f aca="false">SUM($F$2:F36)</f>
-        <v>0.874332</v>
+        <v>0.880014</v>
       </c>
       <c r="H36" s="4"/>
       <c r="I36" s="5" t="n">
-        <v>14.5</v>
+        <v>17.9322</v>
       </c>
       <c r="J36" s="4" t="n">
-        <v>3.5</v>
+        <v>6.49</v>
       </c>
       <c r="K36" s="5"/>
       <c r="L36" s="6" t="n">
-        <v>1.4202</v>
+        <v>1.447</v>
       </c>
       <c r="M36" s="5" t="str">
         <f aca="false">IF(AND(N(K36)&gt;0,N(L36)&gt;0),K36/L36,"")</f>
         <v/>
       </c>
       <c r="N36" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3012,41 +3018,41 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="D37" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D37" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>112</v>
-      </c>
       <c r="F37" s="3" t="n">
-        <v>0.006311</v>
+        <v>0.005833</v>
       </c>
       <c r="G37" s="3" t="n">
         <f aca="false">SUM($F$2:F37)</f>
-        <v>0.880643</v>
+        <v>0.885847</v>
       </c>
       <c r="H37" s="4"/>
       <c r="I37" s="5" t="n">
-        <v>268.9375</v>
+        <v>14.5</v>
       </c>
       <c r="J37" s="4" t="n">
-        <v>0.16</v>
+        <v>3.5</v>
       </c>
       <c r="K37" s="5"/>
       <c r="L37" s="6" t="n">
-        <v>6.8972</v>
+        <v>1.4202</v>
       </c>
       <c r="M37" s="5" t="str">
         <f aca="false">IF(AND(N(K37)&gt;0,N(L37)&gt;0),K37/L37,"")</f>
         <v/>
       </c>
       <c r="N37" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3060,33 +3066,35 @@
         <v>122</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>38</v>
+        <v>114</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>0.006093</v>
+        <v>0.005833</v>
       </c>
       <c r="G38" s="3" t="n">
         <f aca="false">SUM($F$2:F38)</f>
-        <v>0.886736</v>
-      </c>
-      <c r="H38" s="4" t="n">
-        <v>16.31</v>
-      </c>
-      <c r="I38" s="5"/>
-      <c r="J38" s="4"/>
-      <c r="K38" s="5" t="n">
-        <v>20.5039</v>
-      </c>
-      <c r="L38" s="6"/>
+        <v>0.89168</v>
+      </c>
+      <c r="H38" s="4"/>
+      <c r="I38" s="5" t="n">
+        <v>268.9375</v>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="K38" s="5"/>
+      <c r="L38" s="6" t="n">
+        <v>6.8972</v>
+      </c>
       <c r="M38" s="5" t="str">
         <f aca="false">IF(AND(N(K38)&gt;0,N(L38)&gt;0),K38/L38,"")</f>
         <v/>
       </c>
       <c r="N38" s="2" t="s">
-        <v>123</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3094,31 +3102,31 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>125</v>
-      </c>
       <c r="D39" s="2" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>0.005984</v>
+        <v>0.005632</v>
       </c>
       <c r="G39" s="3" t="n">
         <f aca="false">SUM($F$2:F39)</f>
-        <v>0.89272</v>
+        <v>0.897312</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>89.78</v>
+        <v>16.31</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="4"/>
       <c r="K39" s="5" t="n">
-        <v>30.5961</v>
+        <v>20.5039</v>
       </c>
       <c r="L39" s="6"/>
       <c r="M39" s="5" t="str">
@@ -3126,7 +3134,7 @@
         <v/>
       </c>
       <c r="N39" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3140,25 +3148,25 @@
         <v>127</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>0.005114</v>
+        <v>0.005532</v>
       </c>
       <c r="G40" s="3" t="n">
         <f aca="false">SUM($F$2:F40)</f>
-        <v>0.897834</v>
+        <v>0.902844</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>5.85</v>
+        <v>89.78</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="4"/>
       <c r="K40" s="5" t="n">
-        <v>1.9244</v>
+        <v>30.5961</v>
       </c>
       <c r="L40" s="6"/>
       <c r="M40" s="5" t="str">
@@ -3166,7 +3174,7 @@
         <v/>
       </c>
       <c r="N40" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3180,25 +3188,25 @@
         <v>129</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>0.005114</v>
+        <v>0.004727</v>
       </c>
       <c r="G41" s="3" t="n">
         <f aca="false">SUM($F$2:F41)</f>
-        <v>0.902948</v>
+        <v>0.907571</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>19.21</v>
+        <v>5.85</v>
       </c>
       <c r="I41" s="5"/>
       <c r="J41" s="4"/>
       <c r="K41" s="5" t="n">
-        <v>1.885</v>
+        <v>1.9244</v>
       </c>
       <c r="L41" s="6"/>
       <c r="M41" s="5" t="str">
@@ -3206,7 +3214,7 @@
         <v/>
       </c>
       <c r="N41" s="2" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3214,10 +3222,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>20</v>
@@ -3226,29 +3234,27 @@
         <v>25</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>0.005005</v>
+        <v>0.004727</v>
       </c>
       <c r="G42" s="3" t="n">
         <f aca="false">SUM($F$2:F42)</f>
-        <v>0.907953</v>
-      </c>
-      <c r="H42" s="4"/>
-      <c r="I42" s="5" t="n">
-        <v>133.9545</v>
-      </c>
-      <c r="J42" s="4" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="K42" s="5"/>
-      <c r="L42" s="6" t="n">
-        <v>5.8058</v>
-      </c>
+        <v>0.912298</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="I42" s="5"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="5" t="n">
+        <v>1.885</v>
+      </c>
+      <c r="L42" s="6"/>
       <c r="M42" s="5" t="str">
         <f aca="false">IF(AND(N(K42)&gt;0,N(L42)&gt;0),K42/L42,"")</f>
         <v/>
       </c>
       <c r="N42" s="2" t="s">
-        <v>42</v>
+        <v>132</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3262,38 +3268,36 @@
         <v>134</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>0.005005</v>
+        <v>0.004626</v>
       </c>
       <c r="G43" s="3" t="n">
         <f aca="false">SUM($F$2:F43)</f>
-        <v>0.912958</v>
-      </c>
-      <c r="H43" s="4" t="n">
-        <v>113.6</v>
-      </c>
+        <v>0.916924</v>
+      </c>
+      <c r="H43" s="4"/>
       <c r="I43" s="5" t="n">
-        <v>66.8235</v>
+        <v>133.9545</v>
       </c>
       <c r="J43" s="4" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="K43" s="5" t="n">
-        <v>1.9308</v>
-      </c>
+        <v>0.22</v>
+      </c>
+      <c r="K43" s="5"/>
       <c r="L43" s="6" t="n">
-        <v>3.3592</v>
-      </c>
-      <c r="M43" s="5" t="n">
+        <v>5.8058</v>
+      </c>
+      <c r="M43" s="5" t="str">
         <f aca="false">IF(AND(N(K43)&gt;0,N(L43)&gt;0),K43/L43,"")</f>
-        <v>0.574779709454632</v>
-      </c>
-      <c r="N43" s="2"/>
+        <v/>
+      </c>
+      <c r="N43" s="2" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="n">
@@ -3306,34 +3310,38 @@
         <v>136</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0.004461</v>
+        <v>0.004626</v>
       </c>
       <c r="G44" s="3" t="n">
         <f aca="false">SUM($F$2:F44)</f>
-        <v>0.917419</v>
-      </c>
-      <c r="H44" s="4"/>
-      <c r="I44" s="5"/>
+        <v>0.92155</v>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>113.6</v>
+      </c>
+      <c r="I44" s="5" t="n">
+        <v>66.8235</v>
+      </c>
       <c r="J44" s="4" t="n">
-        <v>-0.31</v>
-      </c>
-      <c r="K44" s="5"/>
+        <v>1.7</v>
+      </c>
+      <c r="K44" s="5" t="n">
+        <v>1.9308</v>
+      </c>
       <c r="L44" s="6" t="n">
-        <v>5.2893</v>
-      </c>
-      <c r="M44" s="5" t="str">
+        <v>3.3592</v>
+      </c>
+      <c r="M44" s="5" t="n">
         <f aca="false">IF(AND(N(K44)&gt;0,N(L44)&gt;0),K44/L44,"")</f>
-        <v/>
-      </c>
-      <c r="N44" s="2" t="s">
-        <v>55</v>
-      </c>
+        <v>0.574779709454632</v>
+      </c>
+      <c r="N44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="n">
@@ -3345,26 +3353,34 @@
       <c r="C45" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
+      <c r="D45" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="F45" s="3" t="n">
-        <v>0.004352</v>
+        <v>0.004124</v>
       </c>
       <c r="G45" s="3" t="n">
         <f aca="false">SUM($F$2:F45)</f>
-        <v>0.921771</v>
+        <v>0.925674</v>
       </c>
       <c r="H45" s="4"/>
       <c r="I45" s="5"/>
-      <c r="J45" s="4"/>
+      <c r="J45" s="4" t="n">
+        <v>-0.31</v>
+      </c>
       <c r="K45" s="5"/>
-      <c r="L45" s="6"/>
+      <c r="L45" s="6" t="n">
+        <v>5.2893</v>
+      </c>
       <c r="M45" s="5" t="str">
         <f aca="false">IF(AND(N(K45)&gt;0,N(L45)&gt;0),K45/L45,"")</f>
         <v/>
       </c>
       <c r="N45" s="2" t="s">
-        <v>139</v>
+        <v>57</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3372,39 +3388,31 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C46" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>109</v>
-      </c>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
       <c r="F46" s="3" t="n">
-        <v>0.004243</v>
+        <v>0.004023</v>
       </c>
       <c r="G46" s="3" t="n">
         <f aca="false">SUM($F$2:F46)</f>
-        <v>0.926014</v>
+        <v>0.929697</v>
       </c>
       <c r="H46" s="4"/>
       <c r="I46" s="5"/>
-      <c r="J46" s="4" t="n">
-        <v>-0.27</v>
-      </c>
+      <c r="J46" s="4"/>
       <c r="K46" s="5"/>
-      <c r="L46" s="6" t="n">
-        <v>23.4414</v>
-      </c>
+      <c r="L46" s="6"/>
       <c r="M46" s="5" t="str">
         <f aca="false">IF(AND(N(K46)&gt;0,N(L46)&gt;0),K46/L46,"")</f>
         <v/>
       </c>
       <c r="N46" s="2" t="s">
-        <v>67</v>
+        <v>141</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3421,116 +3429,114 @@
         <v>16</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>144</v>
+        <v>111</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>0.004134</v>
+        <v>0.003922</v>
       </c>
       <c r="G47" s="3" t="n">
         <f aca="false">SUM($F$2:F47)</f>
-        <v>0.930148</v>
-      </c>
-      <c r="H47" s="4" t="n">
-        <v>32.99</v>
-      </c>
-      <c r="I47" s="5" t="n">
-        <v>39.2738</v>
-      </c>
+        <v>0.933619</v>
+      </c>
+      <c r="H47" s="4"/>
+      <c r="I47" s="5"/>
       <c r="J47" s="4" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="K47" s="5" t="n">
-        <v>1.5003</v>
-      </c>
+        <v>-0.27</v>
+      </c>
+      <c r="K47" s="5"/>
       <c r="L47" s="6" t="n">
-        <v>1.2035</v>
-      </c>
-      <c r="M47" s="5" t="n">
+        <v>23.4414</v>
+      </c>
+      <c r="M47" s="5" t="str">
         <f aca="false">IF(AND(N(K47)&gt;0,N(L47)&gt;0),K47/L47,"")</f>
-        <v>1.2466140423764</v>
-      </c>
-      <c r="N47" s="2"/>
+        <v/>
+      </c>
+      <c r="N47" s="2" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="n">
         <v>47</v>
       </c>
       <c r="B48" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="D48" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E48" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>147</v>
-      </c>
       <c r="F48" s="3" t="n">
-        <v>0.004026</v>
+        <v>0.003822</v>
       </c>
       <c r="G48" s="3" t="n">
         <f aca="false">SUM($F$2:F48)</f>
-        <v>0.934174</v>
-      </c>
-      <c r="H48" s="4"/>
-      <c r="I48" s="5"/>
+        <v>0.937441</v>
+      </c>
+      <c r="H48" s="4" t="n">
+        <v>32.99</v>
+      </c>
+      <c r="I48" s="5" t="n">
+        <v>39.2738</v>
+      </c>
       <c r="J48" s="4" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="K48" s="5"/>
+        <v>0.84</v>
+      </c>
+      <c r="K48" s="5" t="n">
+        <v>1.5003</v>
+      </c>
       <c r="L48" s="6" t="n">
-        <v>10.8334</v>
-      </c>
-      <c r="M48" s="5" t="str">
+        <v>1.2035</v>
+      </c>
+      <c r="M48" s="5" t="n">
         <f aca="false">IF(AND(N(K48)&gt;0,N(L48)&gt;0),K48/L48,"")</f>
-        <v/>
-      </c>
-      <c r="N48" s="2" t="s">
-        <v>67</v>
-      </c>
+        <v>1.2466140423764</v>
+      </c>
+      <c r="N48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="n">
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>149</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>29</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>58</v>
+        <v>149</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>0.003699</v>
+        <v>0.003721</v>
       </c>
       <c r="G49" s="3" t="n">
         <f aca="false">SUM($F$2:F49)</f>
-        <v>0.937873</v>
+        <v>0.941162</v>
       </c>
       <c r="H49" s="4"/>
-      <c r="I49" s="5" t="n">
-        <v>81.9595</v>
-      </c>
+      <c r="I49" s="5"/>
       <c r="J49" s="4" t="n">
-        <v>1.73</v>
+        <v>-0.47</v>
       </c>
       <c r="K49" s="5"/>
       <c r="L49" s="6" t="n">
-        <v>11.6272</v>
+        <v>10.8334</v>
       </c>
       <c r="M49" s="5" t="str">
         <f aca="false">IF(AND(N(K49)&gt;0,N(L49)&gt;0),K49/L49,"")</f>
         <v/>
       </c>
       <c r="N49" s="2" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3544,35 +3550,35 @@
         <v>151</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>0.003699</v>
+        <v>0.003419</v>
       </c>
       <c r="G50" s="3" t="n">
         <f aca="false">SUM($F$2:F50)</f>
-        <v>0.941572</v>
+        <v>0.944581</v>
       </c>
       <c r="H50" s="4"/>
       <c r="I50" s="5" t="n">
-        <v>527.027</v>
+        <v>81.9595</v>
       </c>
       <c r="J50" s="4" t="n">
-        <v>0.37</v>
+        <v>1.73</v>
       </c>
       <c r="K50" s="5"/>
       <c r="L50" s="6" t="n">
-        <v>5.807</v>
+        <v>11.6272</v>
       </c>
       <c r="M50" s="5" t="str">
         <f aca="false">IF(AND(N(K50)&gt;0,N(L50)&gt;0),K50/L50,"")</f>
         <v/>
       </c>
       <c r="N50" s="2" t="s">
-        <v>152</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3580,39 +3586,41 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>154</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>112</v>
+        <v>25</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0.003699</v>
+        <v>0.003419</v>
       </c>
       <c r="G51" s="3" t="n">
         <f aca="false">SUM($F$2:F51)</f>
-        <v>0.945271</v>
+        <v>0.948</v>
       </c>
       <c r="H51" s="4"/>
-      <c r="I51" s="5"/>
+      <c r="I51" s="5" t="n">
+        <v>527.027</v>
+      </c>
       <c r="J51" s="4" t="n">
-        <v>-288.2</v>
+        <v>0.37</v>
       </c>
       <c r="K51" s="5"/>
       <c r="L51" s="6" t="n">
-        <v>42.8464</v>
+        <v>5.807</v>
       </c>
       <c r="M51" s="5" t="str">
         <f aca="false">IF(AND(N(K51)&gt;0,N(L51)&gt;0),K51/L51,"")</f>
         <v/>
       </c>
       <c r="N51" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3620,43 +3628,39 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="C52" s="2" t="s">
-        <v>157</v>
-      </c>
       <c r="D52" s="2" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>147</v>
+        <v>114</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>0.003264</v>
+        <v>0.003419</v>
       </c>
       <c r="G52" s="3" t="n">
         <f aca="false">SUM($F$2:F52)</f>
-        <v>0.948535</v>
-      </c>
-      <c r="H52" s="4" t="n">
-        <v>22.69</v>
-      </c>
+        <v>0.951419</v>
+      </c>
+      <c r="H52" s="4"/>
       <c r="I52" s="5"/>
       <c r="J52" s="4" t="n">
-        <v>-0.14</v>
-      </c>
-      <c r="K52" s="5" t="n">
-        <v>1.1335</v>
-      </c>
+        <v>-288.2</v>
+      </c>
+      <c r="K52" s="5"/>
       <c r="L52" s="6" t="n">
-        <v>35.5877</v>
-      </c>
-      <c r="M52" s="5" t="n">
+        <v>42.8464</v>
+      </c>
+      <c r="M52" s="5" t="str">
         <f aca="false">IF(AND(N(K52)&gt;0,N(L52)&gt;0),K52/L52,"")</f>
-        <v>0.0318508923026776</v>
+        <v/>
       </c>
       <c r="N52" s="2" t="s">
-        <v>39</v>
+        <v>157</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3670,33 +3674,37 @@
         <v>159</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>61</v>
+        <v>149</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>0.003155</v>
+        <v>0.003017</v>
       </c>
       <c r="G53" s="3" t="n">
         <f aca="false">SUM($F$2:F53)</f>
-        <v>0.95169</v>
-      </c>
-      <c r="H53" s="4"/>
+        <v>0.954436</v>
+      </c>
+      <c r="H53" s="4" t="n">
+        <v>22.69</v>
+      </c>
       <c r="I53" s="5"/>
       <c r="J53" s="4" t="n">
-        <v>-1.81</v>
-      </c>
-      <c r="K53" s="5"/>
+        <v>-0.14</v>
+      </c>
+      <c r="K53" s="5" t="n">
+        <v>1.1335</v>
+      </c>
       <c r="L53" s="6" t="n">
-        <v>7.3114</v>
-      </c>
-      <c r="M53" s="5" t="str">
+        <v>35.5877</v>
+      </c>
+      <c r="M53" s="5" t="n">
         <f aca="false">IF(AND(N(K53)&gt;0,N(L53)&gt;0),K53/L53,"")</f>
-        <v/>
+        <v>0.0318508923026776</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>67</v>
+        <v>42</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3709,26 +3717,34 @@
       <c r="C54" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
+      <c r="D54" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>63</v>
+      </c>
       <c r="F54" s="3" t="n">
-        <v>0.003046</v>
+        <v>0.002917</v>
       </c>
       <c r="G54" s="3" t="n">
         <f aca="false">SUM($F$2:F54)</f>
-        <v>0.954736</v>
+        <v>0.957353</v>
       </c>
       <c r="H54" s="4"/>
       <c r="I54" s="5"/>
-      <c r="J54" s="4"/>
+      <c r="J54" s="4" t="n">
+        <v>-1.81</v>
+      </c>
       <c r="K54" s="5"/>
-      <c r="L54" s="6"/>
+      <c r="L54" s="6" t="n">
+        <v>7.3114</v>
+      </c>
       <c r="M54" s="5" t="str">
         <f aca="false">IF(AND(N(K54)&gt;0,N(L54)&gt;0),K54/L54,"")</f>
         <v/>
       </c>
       <c r="N54" s="2" t="s">
-        <v>139</v>
+        <v>69</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3745,14 +3761,14 @@
         <v>29</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>0.002829</v>
+        <v>0.002615</v>
       </c>
       <c r="G55" s="3" t="n">
         <f aca="false">SUM($F$2:F55)</f>
-        <v>0.957565</v>
+        <v>0.959968</v>
       </c>
       <c r="H55" s="4"/>
       <c r="I55" s="5"/>
@@ -3768,7 +3784,7 @@
         <v/>
       </c>
       <c r="N55" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3788,11 +3804,11 @@
         <v>25</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>0.002829</v>
+        <v>0.002615</v>
       </c>
       <c r="G56" s="3" t="n">
         <f aca="false">SUM($F$2:F56)</f>
-        <v>0.960394</v>
+        <v>0.962583</v>
       </c>
       <c r="H56" s="4"/>
       <c r="I56" s="5"/>
@@ -3808,7 +3824,7 @@
         <v/>
       </c>
       <c r="N56" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3825,14 +3841,14 @@
         <v>16</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>0.002829</v>
+        <v>0.002615</v>
       </c>
       <c r="G57" s="3" t="n">
         <f aca="false">SUM($F$2:F57)</f>
-        <v>0.963223</v>
+        <v>0.965198</v>
       </c>
       <c r="H57" s="4" t="n">
         <v>18.09</v>
@@ -3852,7 +3868,7 @@
         <v>0.337352160665728</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3869,14 +3885,14 @@
         <v>29</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>0.002829</v>
+        <v>0.002615</v>
       </c>
       <c r="G58" s="3" t="n">
         <f aca="false">SUM($F$2:F58)</f>
-        <v>0.966052</v>
+        <v>0.967813</v>
       </c>
       <c r="H58" s="4"/>
       <c r="I58" s="5"/>
@@ -3892,7 +3908,7 @@
         <v/>
       </c>
       <c r="N58" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3912,11 +3928,11 @@
         <v>25</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>0.002611</v>
+        <v>0.002414</v>
       </c>
       <c r="G59" s="3" t="n">
         <f aca="false">SUM($F$2:F59)</f>
-        <v>0.968663</v>
+        <v>0.970227</v>
       </c>
       <c r="H59" s="4"/>
       <c r="I59" s="5" t="n">
@@ -3934,7 +3950,7 @@
         <v/>
       </c>
       <c r="N59" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3954,11 +3970,11 @@
         <v>25</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>0.002611</v>
+        <v>0.002414</v>
       </c>
       <c r="G60" s="3" t="n">
         <f aca="false">SUM($F$2:F60)</f>
-        <v>0.971274</v>
+        <v>0.972641</v>
       </c>
       <c r="H60" s="4"/>
       <c r="I60" s="5" t="n">
@@ -3976,7 +3992,7 @@
         <v/>
       </c>
       <c r="N60" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3989,27 +4005,39 @@
       <c r="C61" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
+      <c r="D61" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="F61" s="3" t="n">
-        <v>0.002502</v>
+        <v>0.002313</v>
       </c>
       <c r="G61" s="3" t="n">
         <f aca="false">SUM($F$2:F61)</f>
-        <v>0.973776</v>
-      </c>
-      <c r="H61" s="4"/>
-      <c r="I61" s="5"/>
-      <c r="J61" s="4"/>
-      <c r="K61" s="5"/>
-      <c r="L61" s="6"/>
-      <c r="M61" s="5" t="str">
+        <v>0.974954</v>
+      </c>
+      <c r="H61" s="4" t="n">
+        <v>374.98</v>
+      </c>
+      <c r="I61" s="5" t="n">
+        <v>31.859</v>
+      </c>
+      <c r="J61" s="4" t="n">
+        <v>11.77</v>
+      </c>
+      <c r="K61" s="5" t="n">
+        <v>11.8761</v>
+      </c>
+      <c r="L61" s="6" t="n">
+        <v>2.7504</v>
+      </c>
+      <c r="M61" s="5" t="n">
         <f aca="false">IF(AND(N(K61)&gt;0,N(L61)&gt;0),K61/L61,"")</f>
-        <v/>
-      </c>
-      <c r="N61" s="2" t="s">
-        <v>139</v>
-      </c>
+        <v>4.3179537521815</v>
+      </c>
+      <c r="N61" s="2"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="n">
@@ -4025,14 +4053,14 @@
         <v>20</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>0.002394</v>
+        <v>0.002213</v>
       </c>
       <c r="G62" s="3" t="n">
         <f aca="false">SUM($F$2:F62)</f>
-        <v>0.97617</v>
+        <v>0.977167</v>
       </c>
       <c r="H62" s="4" t="n">
         <v>16.44</v>
@@ -4072,11 +4100,11 @@
         <v>25</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>0.002067</v>
+        <v>0.001911</v>
       </c>
       <c r="G63" s="3" t="n">
         <f aca="false">SUM($F$2:F63)</f>
-        <v>0.978237</v>
+        <v>0.979078</v>
       </c>
       <c r="H63" s="4"/>
       <c r="I63" s="5" t="n">
@@ -4114,11 +4142,11 @@
         <v>25</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>0.001958</v>
+        <v>0.00181</v>
       </c>
       <c r="G64" s="3" t="n">
         <f aca="false">SUM($F$2:F64)</f>
-        <v>0.980195</v>
+        <v>0.980888</v>
       </c>
       <c r="H64" s="4"/>
       <c r="I64" s="5"/>
@@ -4134,7 +4162,7 @@
         <v/>
       </c>
       <c r="N64" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4148,17 +4176,17 @@
         <v>183</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>0.001958</v>
+        <v>0.00181</v>
       </c>
       <c r="G65" s="3" t="n">
         <f aca="false">SUM($F$2:F65)</f>
-        <v>0.982153</v>
+        <v>0.982698</v>
       </c>
       <c r="H65" s="4" t="n">
         <v>10.29</v>
@@ -4174,7 +4202,7 @@
         <v/>
       </c>
       <c r="N65" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4194,11 +4222,11 @@
         <v>25</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>0.00185</v>
+        <v>0.00171</v>
       </c>
       <c r="G66" s="3" t="n">
         <f aca="false">SUM($F$2:F66)</f>
-        <v>0.984003</v>
+        <v>0.984408</v>
       </c>
       <c r="H66" s="4"/>
       <c r="I66" s="5" t="n">
@@ -4216,7 +4244,7 @@
         <v/>
       </c>
       <c r="N66" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4236,11 +4264,11 @@
         <v>188</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>0.001741</v>
+        <v>0.001609</v>
       </c>
       <c r="G67" s="3" t="n">
         <f aca="false">SUM($F$2:F67)</f>
-        <v>0.985744</v>
+        <v>0.986017</v>
       </c>
       <c r="H67" s="4" t="n">
         <v>2.97</v>
@@ -4260,7 +4288,7 @@
         <v>0.0071515681115443</v>
       </c>
       <c r="N67" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4280,11 +4308,11 @@
         <v>25</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>0.001741</v>
+        <v>0.001609</v>
       </c>
       <c r="G68" s="3" t="n">
         <f aca="false">SUM($F$2:F68)</f>
-        <v>0.987485</v>
+        <v>0.987626</v>
       </c>
       <c r="H68" s="4"/>
       <c r="I68" s="5"/>
@@ -4300,7 +4328,7 @@
         <v/>
       </c>
       <c r="N68" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4316,11 +4344,11 @@
       <c r="D69" s="2"/>
       <c r="E69" s="2"/>
       <c r="F69" s="3" t="n">
-        <v>0.001632</v>
+        <v>0.001509</v>
       </c>
       <c r="G69" s="3" t="n">
         <f aca="false">SUM($F$2:F69)</f>
-        <v>0.989117</v>
+        <v>0.989135</v>
       </c>
       <c r="H69" s="4"/>
       <c r="I69" s="5"/>
@@ -4332,7 +4360,7 @@
         <v/>
       </c>
       <c r="N69" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4352,11 +4380,11 @@
         <v>17</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>0.001632</v>
+        <v>0.001509</v>
       </c>
       <c r="G70" s="3" t="n">
         <f aca="false">SUM($F$2:F70)</f>
-        <v>0.990749</v>
+        <v>0.990644</v>
       </c>
       <c r="H70" s="4"/>
       <c r="I70" s="5"/>
@@ -4372,7 +4400,7 @@
         <v/>
       </c>
       <c r="N70" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4388,11 +4416,11 @@
       <c r="D71" s="2"/>
       <c r="E71" s="2"/>
       <c r="F71" s="3" t="n">
-        <v>0.001523</v>
+        <v>0.001408</v>
       </c>
       <c r="G71" s="3" t="n">
         <f aca="false">SUM($F$2:F71)</f>
-        <v>0.992272</v>
+        <v>0.992052</v>
       </c>
       <c r="H71" s="4"/>
       <c r="I71" s="5"/>
@@ -4404,7 +4432,7 @@
         <v/>
       </c>
       <c r="N71" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4421,14 +4449,14 @@
         <v>29</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>0.001306</v>
+        <v>0.001207</v>
       </c>
       <c r="G72" s="3" t="n">
         <f aca="false">SUM($F$2:F72)</f>
-        <v>0.993578</v>
+        <v>0.993259</v>
       </c>
       <c r="H72" s="4" t="n">
         <v>144.43</v>
@@ -4468,11 +4496,11 @@
         <v>25</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>0.001197</v>
+        <v>0.001106</v>
       </c>
       <c r="G73" s="3" t="n">
         <f aca="false">SUM($F$2:F73)</f>
-        <v>0.994775</v>
+        <v>0.994365</v>
       </c>
       <c r="H73" s="4"/>
       <c r="I73" s="5"/>
@@ -4488,7 +4516,7 @@
         <v/>
       </c>
       <c r="N73" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4508,11 +4536,11 @@
         <v>25</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>0.001088</v>
+        <v>0.001006</v>
       </c>
       <c r="G74" s="3" t="n">
         <f aca="false">SUM($F$2:F74)</f>
-        <v>0.995863</v>
+        <v>0.995371</v>
       </c>
       <c r="H74" s="4"/>
       <c r="I74" s="5" t="n">
@@ -4550,11 +4578,11 @@
         <v>205</v>
       </c>
       <c r="F75" s="3" t="n">
-        <v>0.001088</v>
+        <v>0.001006</v>
       </c>
       <c r="G75" s="3" t="n">
         <f aca="false">SUM($F$2:F75)</f>
-        <v>0.996951</v>
+        <v>0.996377</v>
       </c>
       <c r="H75" s="4" t="n">
         <v>4.31</v>
@@ -4574,7 +4602,7 @@
         <v>0.00779080530700401</v>
       </c>
       <c r="N75" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4587,39 +4615,27 @@
       <c r="C76" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="D76" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="D76" s="2"/>
+      <c r="E76" s="2"/>
       <c r="F76" s="3" t="n">
-        <v>0.00087</v>
+        <v>0.000805</v>
       </c>
       <c r="G76" s="3" t="n">
         <f aca="false">SUM($F$2:F76)</f>
-        <v>0.997821</v>
-      </c>
-      <c r="H76" s="4" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="I76" s="5" t="n">
-        <v>23.5714</v>
-      </c>
-      <c r="J76" s="4" t="n">
-        <v>0.07</v>
-      </c>
-      <c r="K76" s="5" t="n">
-        <v>0.3714</v>
-      </c>
-      <c r="L76" s="6" t="n">
-        <v>68.9215</v>
-      </c>
-      <c r="M76" s="5" t="n">
+        <v>0.997182</v>
+      </c>
+      <c r="H76" s="4"/>
+      <c r="I76" s="5"/>
+      <c r="J76" s="4"/>
+      <c r="K76" s="5"/>
+      <c r="L76" s="6"/>
+      <c r="M76" s="5" t="str">
         <f aca="false">IF(AND(N(K76)&gt;0,N(L76)&gt;0),K76/L76,"")</f>
-        <v>0.00538873936289837</v>
-      </c>
-      <c r="N76" s="2"/>
+        <v/>
+      </c>
+      <c r="N76" s="2" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="n">
@@ -4635,31 +4651,35 @@
         <v>20</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>112</v>
+        <v>25</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>0.000762</v>
+        <v>0.000805</v>
       </c>
       <c r="G77" s="3" t="n">
         <f aca="false">SUM($F$2:F77)</f>
-        <v>0.998583</v>
+        <v>0.997987</v>
       </c>
       <c r="H77" s="4" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="I77" s="5"/>
-      <c r="J77" s="4"/>
+        <v>1.65</v>
+      </c>
+      <c r="I77" s="5" t="n">
+        <v>23.5714</v>
+      </c>
+      <c r="J77" s="4" t="n">
+        <v>0.07</v>
+      </c>
       <c r="K77" s="5" t="n">
-        <v>0.3474</v>
-      </c>
-      <c r="L77" s="6"/>
-      <c r="M77" s="5" t="str">
+        <v>0.3714</v>
+      </c>
+      <c r="L77" s="6" t="n">
+        <v>68.9215</v>
+      </c>
+      <c r="M77" s="5" t="n">
         <f aca="false">IF(AND(N(K77)&gt;0,N(L77)&gt;0),K77/L77,"")</f>
-        <v/>
-      </c>
-      <c r="N77" s="2" t="s">
-        <v>123</v>
-      </c>
+        <v>0.00538873936289837</v>
+      </c>
+      <c r="N77" s="2"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="n">
@@ -4671,26 +4691,34 @@
       <c r="C78" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
+      <c r="D78" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="F78" s="3" t="n">
-        <v>0.000653</v>
+        <v>0.000704</v>
       </c>
       <c r="G78" s="3" t="n">
         <f aca="false">SUM($F$2:F78)</f>
-        <v>0.999236</v>
-      </c>
-      <c r="H78" s="4"/>
+        <v>0.998691</v>
+      </c>
+      <c r="H78" s="4" t="n">
+        <v>4.58</v>
+      </c>
       <c r="I78" s="5"/>
       <c r="J78" s="4"/>
-      <c r="K78" s="5"/>
+      <c r="K78" s="5" t="n">
+        <v>0.3474</v>
+      </c>
       <c r="L78" s="6"/>
       <c r="M78" s="5" t="str">
         <f aca="false">IF(AND(N(K78)&gt;0,N(L78)&gt;0),K78/L78,"")</f>
         <v/>
       </c>
       <c r="N78" s="2" t="s">
-        <v>74</v>
+        <v>125</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4703,36 +4731,26 @@
       <c r="C79" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="D79" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E79" s="2" t="s">
-        <v>109</v>
-      </c>
+      <c r="D79" s="2"/>
+      <c r="E79" s="2"/>
       <c r="F79" s="3" t="n">
-        <v>0.000544</v>
+        <v>0.000603</v>
       </c>
       <c r="G79" s="3" t="n">
         <f aca="false">SUM($F$2:F79)</f>
-        <v>0.99978</v>
+        <v>0.999294</v>
       </c>
       <c r="H79" s="4"/>
-      <c r="I79" s="5" t="n">
-        <v>326.3889</v>
-      </c>
-      <c r="J79" s="4" t="n">
-        <v>0.72</v>
-      </c>
+      <c r="I79" s="5"/>
+      <c r="J79" s="4"/>
       <c r="K79" s="5"/>
-      <c r="L79" s="6" t="n">
-        <v>12.8107</v>
-      </c>
+      <c r="L79" s="6"/>
       <c r="M79" s="5" t="str">
         <f aca="false">IF(AND(N(K79)&gt;0,N(L79)&gt;0),K79/L79,"")</f>
         <v/>
       </c>
       <c r="N79" s="2" t="s">
-        <v>26</v>
+        <v>76</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4746,37 +4764,79 @@
         <v>215</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>188</v>
+        <v>111</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>0.000218</v>
+        <v>0.000503</v>
       </c>
       <c r="G80" s="3" t="n">
         <f aca="false">SUM($F$2:F80)</f>
-        <v>0.999998</v>
+        <v>0.999797</v>
       </c>
       <c r="H80" s="4"/>
-      <c r="I80" s="5"/>
+      <c r="I80" s="5" t="n">
+        <v>326.3889</v>
+      </c>
       <c r="J80" s="4" t="n">
-        <v>-1.16</v>
+        <v>0.72</v>
       </c>
       <c r="K80" s="5"/>
       <c r="L80" s="6" t="n">
-        <v>1.0428</v>
+        <v>12.8107</v>
       </c>
       <c r="M80" s="5" t="str">
         <f aca="false">IF(AND(N(K80)&gt;0,N(L80)&gt;0),K80/L80,"")</f>
         <v/>
       </c>
       <c r="N80" s="2" t="s">
-        <v>67</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F81" s="3" t="n">
+        <v>0.000201</v>
+      </c>
+      <c r="G81" s="3" t="n">
+        <f aca="false">SUM($F$2:F81)</f>
+        <v>0.999998</v>
+      </c>
+      <c r="H81" s="4"/>
+      <c r="I81" s="5"/>
+      <c r="J81" s="4" t="n">
+        <v>-1.16</v>
+      </c>
+      <c r="K81" s="5"/>
+      <c r="L81" s="6" t="n">
+        <v>1.0428</v>
+      </c>
+      <c r="M81" s="5" t="str">
+        <f aca="false">IF(AND(N(K81)&gt;0,N(L81)&gt;0),K81/L81,"")</f>
+        <v/>
+      </c>
+      <c r="N81" s="2" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N80"/>
+  <autoFilter ref="A1:N81"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4807,97 +4867,97 @@
         <v>3</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="3" t="n">
-        <f aca="false">SUMIF(Holdings!$D$2:$D$80,A2,Holdings!$F$2:$F$80)</f>
-        <v>0.027962</v>
+        <f aca="false">SUMIF(Holdings!$D$2:$D$81,A2,Holdings!$F$2:$F$81)</f>
+        <v>0.025848</v>
       </c>
       <c r="C2" s="2" t="n">
-        <f aca="false">COUNTIF(Holdings!$D$2:$D$80,A2)</f>
+        <f aca="false">COUNTIF(Holdings!$D$2:$D$81,A2)</f>
         <v>2</v>
       </c>
       <c r="D2" s="8" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$80,Holdings!$D$2:$D$80,A2,Holdings!$I$2:$I$80,"&lt;=100"),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$81,Holdings!$D$2:$D$81,A2,Holdings!$I$2:$I$81,"&lt;=100"),"")</f>
         <v>16.9338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B3" s="3" t="n">
-        <f aca="false">SUMIF(Holdings!$D$2:$D$80,A3,Holdings!$F$2:$F$80)</f>
-        <v>0.066804</v>
+        <f aca="false">SUMIF(Holdings!$D$2:$D$81,A3,Holdings!$F$2:$F$81)</f>
+        <v>0.061751</v>
       </c>
       <c r="C3" s="2" t="n">
-        <f aca="false">COUNTIF(Holdings!$D$2:$D$80,A3)</f>
+        <f aca="false">COUNTIF(Holdings!$D$2:$D$81,A3)</f>
         <v>5</v>
       </c>
       <c r="D3" s="8" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$80,Holdings!$D$2:$D$80,A3,Holdings!$I$2:$I$80,"&lt;=100"),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$81,Holdings!$D$2:$D$81,A3,Holdings!$I$2:$I$81,"&lt;=100"),"")</f>
         <v>14.5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B4" s="3" t="n">
-        <f aca="false">SUMIF(Holdings!$D$2:$D$80,A4,Holdings!$F$2:$F$80)</f>
+        <f aca="false">SUMIF(Holdings!$D$2:$D$81,A4,Holdings!$F$2:$F$81)</f>
         <v>0</v>
       </c>
       <c r="C4" s="2" t="n">
-        <f aca="false">COUNTIF(Holdings!$D$2:$D$80,A4)</f>
+        <f aca="false">COUNTIF(Holdings!$D$2:$D$81,A4)</f>
         <v>0</v>
       </c>
       <c r="D4" s="8" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$80,Holdings!$D$2:$D$80,A4,Holdings!$I$2:$I$80,"&lt;=100"),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$81,Holdings!$D$2:$D$81,A4,Holdings!$I$2:$I$81,"&lt;=100"),"")</f>
         <v/>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B5" s="3" t="n">
-        <f aca="false">SUMIF(Holdings!$D$2:$D$80,A5,Holdings!$F$2:$F$80)</f>
+        <f aca="false">SUMIF(Holdings!$D$2:$D$81,A5,Holdings!$F$2:$F$81)</f>
         <v>0</v>
       </c>
       <c r="C5" s="2" t="n">
-        <f aca="false">COUNTIF(Holdings!$D$2:$D$80,A5)</f>
+        <f aca="false">COUNTIF(Holdings!$D$2:$D$81,A5)</f>
         <v>0</v>
       </c>
       <c r="D5" s="8" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$80,Holdings!$D$2:$D$80,A5,Holdings!$I$2:$I$80,"&lt;=100"),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$81,Holdings!$D$2:$D$81,A5,Holdings!$I$2:$I$81,"&lt;=100"),"")</f>
         <v/>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B6" s="3" t="n">
-        <f aca="false">SUMIF(Holdings!$D$2:$D$80,A6,Holdings!$F$2:$F$80)</f>
+        <f aca="false">SUMIF(Holdings!$D$2:$D$81,A6,Holdings!$F$2:$F$81)</f>
         <v>0</v>
       </c>
       <c r="C6" s="2" t="n">
-        <f aca="false">COUNTIF(Holdings!$D$2:$D$80,A6)</f>
+        <f aca="false">COUNTIF(Holdings!$D$2:$D$81,A6)</f>
         <v>0</v>
       </c>
       <c r="D6" s="8" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$80,Holdings!$D$2:$D$80,A6,Holdings!$I$2:$I$80,"&lt;=100"),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$81,Holdings!$D$2:$D$81,A6,Holdings!$I$2:$I$81,"&lt;=100"),"")</f>
         <v/>
       </c>
     </row>
@@ -4906,15 +4966,15 @@
         <v>16</v>
       </c>
       <c r="B7" s="3" t="n">
-        <f aca="false">SUMIF(Holdings!$D$2:$D$80,A7,Holdings!$F$2:$F$80)</f>
-        <v>0.12077</v>
+        <f aca="false">SUMIF(Holdings!$D$2:$D$81,A7,Holdings!$F$2:$F$81)</f>
+        <v>0.111637</v>
       </c>
       <c r="C7" s="2" t="n">
-        <f aca="false">COUNTIF(Holdings!$D$2:$D$80,A7)</f>
+        <f aca="false">COUNTIF(Holdings!$D$2:$D$81,A7)</f>
         <v>8</v>
       </c>
       <c r="D7" s="8" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$80,Holdings!$D$2:$D$80,A7,Holdings!$I$2:$I$80,"&lt;=100"),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$81,Holdings!$D$2:$D$81,A7,Holdings!$I$2:$I$81,"&lt;=100"),"")</f>
         <v>42.44905</v>
       </c>
     </row>
@@ -4923,16 +4983,16 @@
         <v>20</v>
       </c>
       <c r="B8" s="3" t="n">
-        <f aca="false">SUMIF(Holdings!$D$2:$D$80,A8,Holdings!$F$2:$F$80)</f>
-        <v>0.527798</v>
+        <f aca="false">SUMIF(Holdings!$D$2:$D$81,A8,Holdings!$F$2:$F$81)</f>
+        <v>0.490193</v>
       </c>
       <c r="C8" s="2" t="n">
-        <f aca="false">COUNTIF(Holdings!$D$2:$D$80,A8)</f>
-        <v>39</v>
+        <f aca="false">COUNTIF(Holdings!$D$2:$D$81,A8)</f>
+        <v>40</v>
       </c>
       <c r="D8" s="8" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$80,Holdings!$D$2:$D$80,A8,Holdings!$I$2:$I$80,"&lt;=100"),"")</f>
-        <v>31.717275</v>
+        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$81,Holdings!$D$2:$D$81,A8,Holdings!$I$2:$I$81,"&lt;=100"),"")</f>
+        <v>31.7256117647059</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4940,86 +5000,86 @@
         <v>29</v>
       </c>
       <c r="B9" s="3" t="n">
-        <f aca="false">SUMIF(Holdings!$D$2:$D$80,A9,Holdings!$F$2:$F$80)</f>
-        <v>0.217061</v>
+        <f aca="false">SUMIF(Holdings!$D$2:$D$81,A9,Holdings!$F$2:$F$81)</f>
+        <v>0.278285</v>
       </c>
       <c r="C9" s="2" t="n">
-        <f aca="false">COUNTIF(Holdings!$D$2:$D$80,A9)</f>
-        <v>17</v>
+        <f aca="false">COUNTIF(Holdings!$D$2:$D$81,A9)</f>
+        <v>18</v>
       </c>
       <c r="D9" s="8" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$80,Holdings!$D$2:$D$80,A9,Holdings!$I$2:$I$80,"&lt;=100"),"")</f>
-        <v>54.2562571428571</v>
+        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$81,Holdings!$D$2:$D$81,A9,Holdings!$I$2:$I$81,"&lt;=100"),"")</f>
+        <v>52.7294875</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B10" s="3" t="n">
-        <f aca="false">SUMIF(Holdings!$D$2:$D$80,A10,Holdings!$F$2:$F$80)</f>
+        <f aca="false">SUMIF(Holdings!$D$2:$D$81,A10,Holdings!$F$2:$F$81)</f>
         <v>0</v>
       </c>
       <c r="C10" s="2" t="n">
-        <f aca="false">COUNTIF(Holdings!$D$2:$D$80,A10)</f>
+        <f aca="false">COUNTIF(Holdings!$D$2:$D$81,A10)</f>
         <v>0</v>
       </c>
       <c r="D10" s="8" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$80,Holdings!$D$2:$D$80,A10,Holdings!$I$2:$I$80,"&lt;=100"),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$81,Holdings!$D$2:$D$81,A10,Holdings!$I$2:$I$81,"&lt;=100"),"")</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B11" s="3" t="n">
-        <f aca="false">SUMIF(Holdings!$D$2:$D$80,A11,Holdings!$F$2:$F$80)</f>
+        <f aca="false">SUMIF(Holdings!$D$2:$D$81,A11,Holdings!$F$2:$F$81)</f>
         <v>0</v>
       </c>
       <c r="C11" s="2" t="n">
-        <f aca="false">COUNTIF(Holdings!$D$2:$D$80,A11)</f>
+        <f aca="false">COUNTIF(Holdings!$D$2:$D$81,A11)</f>
         <v>0</v>
       </c>
       <c r="D11" s="8" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$80,Holdings!$D$2:$D$80,A11,Holdings!$I$2:$I$80,"&lt;=100"),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$81,Holdings!$D$2:$D$81,A11,Holdings!$I$2:$I$81,"&lt;=100"),"")</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B12" s="3" t="n">
-        <f aca="false">SUMIF(Holdings!$D$2:$D$80,A12,Holdings!$F$2:$F$80)</f>
+        <f aca="false">SUMIF(Holdings!$D$2:$D$81,A12,Holdings!$F$2:$F$81)</f>
         <v>0</v>
       </c>
       <c r="C12" s="2" t="n">
-        <f aca="false">COUNTIF(Holdings!$D$2:$D$80,A12)</f>
+        <f aca="false">COUNTIF(Holdings!$D$2:$D$81,A12)</f>
         <v>0</v>
       </c>
       <c r="D12" s="8" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$80,Holdings!$D$2:$D$80,A12,Holdings!$I$2:$I$80,"&lt;=100"),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS(Holdings!$I$2:$I$81,Holdings!$D$2:$D$81,A12,Holdings!$I$2:$I$81,"&lt;=100"),"")</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B13" s="3" t="n">
         <f aca="false">1-SUM(B2:B12)</f>
-        <v>0.0396050000000001</v>
+        <v>0.032286</v>
       </c>
       <c r="C13" s="2" t="n">
-        <f aca="false">COUNTBLANK(Holdings!$D$2:$D$80)</f>
-        <v>8</v>
+        <f aca="false">COUNTBLANK(Holdings!$D$2:$D$81)</f>
+        <v>7</v>
       </c>
       <c r="D13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B14" s="10" t="n">
         <f aca="false">SUM(B2:B13)</f>
@@ -5027,7 +5087,7 @@
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">SUM(C2:C13)</f>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D14" s="11"/>
     </row>
@@ -5056,25 +5116,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B3" s="14" t="n">
-        <v>0.2543</v>
+        <v>0.235</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B4" s="15" t="n">
         <v>0.135</v>
@@ -5085,13 +5145,13 @@
         <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5099,14 +5159,14 @@
         <v>14</v>
       </c>
       <c r="B7" s="16" t="n">
-        <v>0.0913</v>
+        <v>0.0844</v>
       </c>
       <c r="C7" s="16" t="n">
         <v>0.002</v>
       </c>
       <c r="D7" s="17" t="n">
         <f aca="false">IF(C7&gt;0,B7/C7,"")</f>
-        <v>45.65</v>
+        <v>42.2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5114,83 +5174,83 @@
         <v>27</v>
       </c>
       <c r="B8" s="16" t="n">
-        <v>0.0862</v>
+        <v>0.0797</v>
       </c>
       <c r="C8" s="16" t="n">
         <v>0.0773</v>
       </c>
       <c r="D8" s="17" t="n">
         <f aca="false">IF(C8&gt;0,B8/C8,"")</f>
-        <v>1.11513583441138</v>
+        <v>1.03104786545925</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B9" s="16" t="n">
-        <v>0.0224</v>
+        <v>0.0207</v>
       </c>
       <c r="C9" s="16" t="n">
         <v>0.0208</v>
       </c>
       <c r="D9" s="17" t="n">
         <f aca="false">IF(C9&gt;0,B9/C9,"")</f>
-        <v>1.07692307692308</v>
+        <v>0.995192307692308</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B10" s="16" t="n">
-        <v>0.022</v>
+        <v>0.0203</v>
       </c>
       <c r="C10" s="16" t="n">
         <v>0.0316</v>
       </c>
       <c r="D10" s="17" t="n">
         <f aca="false">IF(C10&gt;0,B10/C10,"")</f>
-        <v>0.69620253164557</v>
+        <v>0.642405063291139</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B11" s="16" t="n">
-        <v>0.0212</v>
+        <v>0.0196</v>
       </c>
       <c r="C11" s="16" t="n">
         <v>0.0026</v>
       </c>
       <c r="D11" s="17" t="n">
         <f aca="false">IF(C11&gt;0,B11/C11,"")</f>
-        <v>8.15384615384616</v>
+        <v>7.53846153846154</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B12" s="16" t="n">
-        <v>0.0112</v>
+        <v>0.0104</v>
       </c>
       <c r="C12" s="16" t="n">
         <v>0.0007</v>
       </c>
       <c r="D12" s="17" t="n">
         <f aca="false">IF(C12&gt;0,B12/C12,"")</f>
-        <v>16</v>
+        <v>14.8571428571429</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B13" s="14" t="n">
         <f aca="false">SUM(B7:B12)</f>
-        <v>0.2543</v>
+        <v>0.2351</v>
       </c>
       <c r="C13" s="15" t="n">
         <f aca="false">SUM(C7:C12)</f>
@@ -5221,42 +5281,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="18" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5264,17 +5324,17 @@
     </row>
     <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -5309,34 +5369,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5665,12 +5725,12 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C13" s="23" t="n">
         <f aca="false">COUNT(A2:A10)</f>
@@ -5679,7 +5739,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C14" s="23" t="n">
         <f aca="false">COUNTIF(D2:D10,"&gt;=0")</f>
@@ -5688,7 +5748,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C15" s="23" t="n">
         <f aca="false">COUNTIF(D2:D10,"&lt;0")</f>
@@ -5697,7 +5757,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C16" s="16" t="n">
         <f aca="false">AVERAGE(D2:D10)</f>
@@ -5706,7 +5766,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C17" s="16" t="n">
         <f aca="false">(H10)^(1/COUNT(A2:A10))-1</f>
@@ -5715,7 +5775,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C18" s="16" t="n">
         <f aca="false">AVERAGE(F2:F10)</f>
@@ -5724,7 +5784,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C19" s="16" t="n">
         <f aca="false">MAX(D2:D10)</f>
@@ -5733,7 +5793,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C20" s="16" t="n">
         <f aca="false">MIN(D2:D10)</f>
@@ -5742,7 +5802,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C21" s="16" t="n">
         <f aca="false">STDEV(D2:D10)</f>
@@ -5751,7 +5811,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C22" s="24" t="n">
         <f aca="false">H10</f>
@@ -5760,7 +5820,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C23" s="16" t="n">
         <f aca="false">AVERAGE(J2:J10)</f>
@@ -5769,7 +5829,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C24" s="16" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+J2:J10)))^(1/COUNT(J2:J10))-1</f>
@@ -5778,7 +5838,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C25" s="24" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+J2:J10)))</f>
@@ -5787,7 +5847,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C26" s="16" t="n">
         <f aca="false">STDEV(J2:J10)</f>
@@ -5796,12 +5856,12 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="25" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="25" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -5839,57 +5899,57 @@
   <sheetData>
     <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C2" s="20" t="n">
         <f aca="false">COUNTIF('Annual Returns'!$B$2:$B$10,"2010s")</f>
@@ -5946,10 +6006,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="20" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C3" s="20" t="n">
         <f aca="false">COUNTIF('Annual Returns'!$B$2:$B$10,"2020s")</f>
@@ -6006,10 +6066,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C4" s="26" t="n">
         <f aca="false">COUNT('Annual Returns'!$A$2:$A$10)</f>
@@ -6066,17 +6126,17 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="25" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="25" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="25" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>